<commit_message>
feat(client): establish Critterarium v1.1.0
- Finalize taxonomy UI and organism research workflows.
- Complete video QA and align all machine-readable version metadata.
</commit_message>
<xml_diff>
--- a/database/plantae-fungi.xlsx
+++ b/database/plantae-fungi.xlsx
@@ -670,22 +670,22 @@
         <v/>
       </c>
       <c r="AD2" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/7/7a/Sunflower_head_2015_G4.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/8/8b/Sunflower_head_2015_G3.jpg</v>
       </c>
       <c r="AE2" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Sunflower_head_2015_G1.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Sunflower_head_2015_G3.jpg</v>
       </c>
       <c r="AF2" t="str">
         <v>Public Domain</v>
       </c>
       <c r="AG2" t="str">
-        <v>https://www.youtube.com/watch?v=5lbup7WTmy8</v>
+        <v>https://www.youtube.com/watch?v=4_PKTESKseg</v>
       </c>
       <c r="AH2" t="str">
-        <v>5lbup7WTmy8</v>
+        <v>4_PKTESKseg</v>
       </c>
       <c r="AI2" t="str">
-        <v>4K Ultra HD Sunflower Fields Beautiful Natural Scenery with Nature Sounds Trailer 2</v>
+        <v>Beautiful sunflower field in summer | Nature Scenery Documentary 4K</v>
       </c>
       <c r="AJ2" t="str">
         <v>4K</v>
@@ -697,7 +697,7 @@
         <v>cozymuseum-foundation | gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM2" t="str">
-        <v>2026-08-01T15:17:24.906Z</v>
+        <v>2026-08-01T16:54:07.789Z</v>
       </c>
       <c r="AN2">
         <v>0.99</v>
@@ -745,10 +745,10 @@
         <v/>
       </c>
       <c r="BC2">
-        <v>4800</v>
+        <v>3400</v>
       </c>
       <c r="BD2">
-        <v>3350</v>
+        <v>4900</v>
       </c>
       <c r="BE2" t="str">
         <v>4K</v>
@@ -852,7 +852,7 @@
         <v/>
       </c>
       <c r="AD3" t="str">
-        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/293129369/original.jpeg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/f/f5/Lotus_flower_%28978659%29.jpg</v>
       </c>
       <c r="AE3" t="str">
         <v>https://commons.wikimedia.org/wiki/File:Lotus_flower_(978659).jpg</v>
@@ -861,13 +861,13 @@
         <v>CC0</v>
       </c>
       <c r="AG3" t="str">
-        <v>https://www.youtube.com/watch?v=mTE1cJWOClQ</v>
+        <v>https://www.youtube.com/watch?v=-WIX_e2KzTI</v>
       </c>
       <c r="AH3" t="str">
-        <v>mTE1cJWOClQ</v>
+        <v>-WIX_e2KzTI</v>
       </c>
       <c r="AI3" t="str">
-        <v>FLYING OVER ELAFONISI (4K UHD) – Soothing Music Along With Beautiful Nature Video -4K Video ULTRA HD</v>
+        <v>Pakistan's Most Beautiful Kanwal (Lotus) Flowers | Nature Documentary</v>
       </c>
       <c r="AJ3" t="str">
         <v>4K</v>
@@ -879,7 +879,7 @@
         <v>cozymuseum-foundation | gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM3" t="str">
-        <v>2026-08-01T15:01:35.462Z</v>
+        <v>2026-08-01T16:54:12.540Z</v>
       </c>
       <c r="AN3">
         <v>0.99</v>
@@ -1043,13 +1043,13 @@
         <v>CC0</v>
       </c>
       <c r="AG4" t="str">
-        <v>https://www.youtube.com/watch?v=FWi2bn40ma4</v>
+        <v>https://www.youtube.com/watch?v=WWtOxnWUmLw</v>
       </c>
       <c r="AH4" t="str">
-        <v>FWi2bn40ma4</v>
+        <v>WWtOxnWUmLw</v>
       </c>
       <c r="AI4" t="str">
-        <v>The Tallest Trees on Earth - 4K Nature Documentary Film | Redwood National and State Parks</v>
+        <v>Ferns | Fern Plants Full Documentary | Amazing Facts about Ferns.</v>
       </c>
       <c r="AJ4" t="str">
         <v>4K</v>
@@ -1061,7 +1061,7 @@
         <v>cozymuseum-foundation | gbif | wikimedia | youtube</v>
       </c>
       <c r="AM4" t="str">
-        <v>2026-08-01T13:51:27.379Z</v>
+        <v>2026-08-01T16:54:15.926Z</v>
       </c>
       <c r="AN4">
         <v>0.94</v>
@@ -1216,22 +1216,22 @@
         <v/>
       </c>
       <c r="AD5" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/a/a3/Bermuda_Maidenhair_Fern-02.JPG</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/147598479/original.jpeg</v>
       </c>
       <c r="AE5" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Bermuda_Maidenhair_Fern-01.JPG</v>
+        <v>https://www.inaturalist.org/photos/147598479</v>
       </c>
       <c r="AF5" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG5" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=ML1wDBYV5us</v>
       </c>
       <c r="AH5" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>ML1wDBYV5us</v>
       </c>
       <c r="AI5" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>Southern Maidenhair Fern | The Nature and Philosophy</v>
       </c>
       <c r="AJ5" t="str">
         <v>4K</v>
@@ -1243,7 +1243,7 @@
         <v>cozymuseum-foundation | gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM5" t="str">
-        <v>2026-08-01T15:17:32.841Z</v>
+        <v>2026-08-01T16:54:19.938Z</v>
       </c>
       <c r="AN5">
         <v>0.92</v>
@@ -1291,16 +1291,16 @@
         <v/>
       </c>
       <c r="BC5">
-        <v>3072</v>
+        <v>2048</v>
       </c>
       <c r="BD5">
-        <v>2304</v>
+        <v>1536</v>
       </c>
       <c r="BE5" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF5" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG5" t="str">
         <v>rights-free</v>
@@ -1401,19 +1401,19 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/439733397/original.jpeg</v>
       </c>
       <c r="AE6" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:AD2009Sep20_Amanita_muscaria_02.jpg</v>
+        <v>https://www.inaturalist.org/photos/439733397</v>
       </c>
       <c r="AF6" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG6" t="str">
-        <v>https://www.youtube.com/watch?v=dBx0KvdhZeA</v>
+        <v>https://www.youtube.com/watch?v=oRNjpNeiZ8Y</v>
       </c>
       <c r="AH6" t="str">
-        <v>dBx0KvdhZeA</v>
+        <v>oRNjpNeiZ8Y</v>
       </c>
       <c r="AI6" t="str">
-        <v>AMANITA SEASON |The Forgotten Secret of our Forests | Soothing Nature in 4K Ultra HD</v>
+        <v>AMANITA MUSCARIA documentary</v>
       </c>
       <c r="AJ6" t="str">
         <v>4K</v>
@@ -1425,7 +1425,7 @@
         <v>cozymuseum-foundation | gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM6" t="str">
-        <v>2026-08-01T15:01:42.875Z</v>
+        <v>2026-08-01T16:54:23.957Z</v>
       </c>
       <c r="AN6">
         <v>0.97</v>
@@ -1473,16 +1473,16 @@
         <v/>
       </c>
       <c r="BC6">
-        <v>3640</v>
+        <v>2048</v>
       </c>
       <c r="BD6">
-        <v>2436</v>
+        <v>1536</v>
       </c>
       <c r="BE6" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF6" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG6" t="str">
         <v>rights-free</v>
@@ -1583,19 +1583,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/7/71/Basswood_small_white_flower_mushroom.jpg</v>
       </c>
       <c r="AE7" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Lentinula_edodes_20101113_d.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Basswood_small_white_flower_mushroom.jpg</v>
       </c>
       <c r="AF7" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG7" t="str">
-        <v>https://www.youtube.com/watch?v=WKoPSlyeMJI</v>
+        <v>https://www.youtube.com/watch?v=xjVU4Poa2p0</v>
       </c>
       <c r="AH7" t="str">
-        <v>WKoPSlyeMJI</v>
+        <v>xjVU4Poa2p0</v>
       </c>
       <c r="AI7" t="str">
-        <v>Exploring Nature’s Secrets with David Attenborough (4K Documentary)</v>
+        <v>Shiitake Documentary -- 4k</v>
       </c>
       <c r="AJ7" t="str">
         <v>4K</v>
@@ -1607,7 +1607,7 @@
         <v>cozymuseum-foundation | gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM7" t="str">
-        <v>2026-08-01T15:17:37.572Z</v>
+        <v>2026-08-01T16:54:27.749Z</v>
       </c>
       <c r="AN7">
         <v>0.98</v>
@@ -1655,16 +1655,16 @@
         <v/>
       </c>
       <c r="BC7">
-        <v>2755</v>
+        <v>3000</v>
       </c>
       <c r="BD7">
-        <v>2066</v>
+        <v>3000</v>
       </c>
       <c r="BE7" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF7" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG7" t="str">
         <v>rights-free</v>
@@ -1765,19 +1765,19 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/243751650/original.jpeg</v>
       </c>
       <c r="AE8" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Hericium_erinaceus_104664221.jpg</v>
+        <v>https://www.inaturalist.org/photos/243751650</v>
       </c>
       <c r="AF8" t="str">
         <v>CC0</v>
       </c>
       <c r="AG8" t="str">
-        <v>https://www.youtube.com/watch?v=bCaW1Aefqa8</v>
+        <v>https://www.youtube.com/watch?v=0ONboSKuqAc</v>
       </c>
       <c r="AH8" t="str">
-        <v>bCaW1Aefqa8</v>
+        <v>0ONboSKuqAc</v>
       </c>
       <c r="AI8" t="str">
-        <v>Monster Of The Arctic: Lion's Mane Jellyfish | 4K Ocean Documentary</v>
+        <v>The Mushroom That Rebuilds Your Brain: Lion’s Mane | Mushroom Documentary</v>
       </c>
       <c r="AJ8" t="str">
         <v>4K</v>
@@ -1789,7 +1789,7 @@
         <v>cozymuseum-foundation | gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM8" t="str">
-        <v>2026-08-01T15:01:47.010Z</v>
+        <v>2026-08-01T16:54:32.900Z</v>
       </c>
       <c r="AN8">
         <v>0.99</v>
@@ -1837,16 +1837,16 @@
         <v/>
       </c>
       <c r="BC8">
+        <v>2048</v>
+      </c>
+      <c r="BD8">
         <v>1536</v>
-      </c>
-      <c r="BD8">
-        <v>2048</v>
       </c>
       <c r="BE8" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF8" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG8" t="str">
         <v>rights-free</v>
@@ -1947,19 +1947,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/1/19/Leitpflanzen_der_palaeozoischen_Steinkohlenablagerungen_in_Mittel-Europa_%28IA_leitpflanzender2hofm%29.pdf</v>
       </c>
       <c r="AE9" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Palaeontographica_(IA_palaeontographic18cass).pdf</v>
+        <v>https://commons.wikimedia.org/wiki/File:Leitpflanzen_der_palaeozoischen_Steinkohlenablagerungen_in_Mittel-Europa_(IA_leitpflanzender2hofm).pdf</v>
       </c>
       <c r="AF9" t="str">
         <v>Public Domain</v>
       </c>
       <c r="AG9" t="str">
-        <v>https://www.youtube.com/watch?v=FWi2bn40ma4</v>
+        <v>https://www.youtube.com/watch?v=95WlXQR30Ls</v>
       </c>
       <c r="AH9" t="str">
-        <v>FWi2bn40ma4</v>
+        <v>95WlXQR30Ls</v>
       </c>
       <c r="AI9" t="str">
-        <v>The Tallest Trees on Earth - 4K Nature Documentary Film | Redwood National and State Parks</v>
+        <v>Dead Trees, Wild Lives: What the Forest Hides | Full Documentary</v>
       </c>
       <c r="AJ9" t="str">
         <v>4K</v>
@@ -1971,7 +1971,7 @@
         <v>gbif | wikipedia | youtube | wikimedia</v>
       </c>
       <c r="AM9" t="str">
-        <v>2026-08-01T15:17:43.025Z</v>
+        <v>2026-08-01T16:54:36.278Z</v>
       </c>
       <c r="AN9">
         <v>0.94</v>
@@ -2019,13 +2019,13 @@
         <v/>
       </c>
       <c r="BC9">
-        <v>1297</v>
+        <v>2891</v>
       </c>
       <c r="BD9">
-        <v>1841</v>
+        <v>1904</v>
       </c>
       <c r="BE9" t="str">
-        <v>HD</v>
+        <v>Full HD</v>
       </c>
       <c r="BF9" t="str">
         <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
@@ -2126,13 +2126,13 @@
         <v/>
       </c>
       <c r="AD10" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/3/33/Verhandlungen_%28IA_verhandlungen140natu%29.pdf</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/3/3f/F%C3%B6ldtani_k%C3%B6zl%C3%B6ny_%28IA_foldtanikozlony1318magy%29.pdf</v>
       </c>
       <c r="AE10" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Glossopteris_sp.,_seed_ferns,_Permian_-_Triassic_-_Houston_Museum_of_Natural_Science_-_DSC01765.JPG</v>
+        <v>https://commons.wikimedia.org/wiki/File:F%C3%B6ldtani_k%C3%B6zl%C3%B6ny_(IA_foldtanikozlony1318magy).pdf</v>
       </c>
       <c r="AF10" t="str">
-        <v>CC0</v>
+        <v>Public Domain</v>
       </c>
       <c r="AG10" t="str">
         <v>https://www.youtube.com/watch?v=Y58UtzZNtyU</v>
@@ -2153,7 +2153,7 @@
         <v>gbif | wikipedia | youtube | wikimedia</v>
       </c>
       <c r="AM10" t="str">
-        <v>2026-08-01T15:17:45.109Z</v>
+        <v>2026-08-01T16:54:39.692Z</v>
       </c>
       <c r="AN10">
         <v>0.99</v>
@@ -2201,16 +2201,16 @@
         <v/>
       </c>
       <c r="BC10">
-        <v>3240</v>
+        <v>979</v>
       </c>
       <c r="BD10">
-        <v>4320</v>
+        <v>1485</v>
       </c>
       <c r="BE10" t="str">
-        <v>4K</v>
+        <v>HD</v>
       </c>
       <c r="BF10" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
       </c>
       <c r="BG10" t="str">
         <v>rights-free</v>
@@ -2308,22 +2308,22 @@
         <v/>
       </c>
       <c r="AD11" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/4/49/Caulerpa_lentillifera_-_National_Museum_of_Nature_and_Science%2C_Tokyo_-_DSC06909.JPG</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/7/73/Punta-Tuna-Beach-Sargassum-Close-Up.jpg</v>
       </c>
       <c r="AE11" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Caulerpa_lentillifera_-_National_Museum_of_Nature_and_Science,_Tokyo_-_DSC06909.JPG</v>
+        <v>https://commons.wikimedia.org/wiki/File:Punta-Tuna-Beach-Sargassum-Close-Up.jpg</v>
       </c>
       <c r="AF11" t="str">
         <v>CC0</v>
       </c>
       <c r="AG11" t="str">
-        <v>https://www.youtube.com/watch?v=mTE1cJWOClQ</v>
+        <v>https://www.youtube.com/watch?v=u0qvrB1GkTo</v>
       </c>
       <c r="AH11" t="str">
-        <v>mTE1cJWOClQ</v>
+        <v>u0qvrB1GkTo</v>
       </c>
       <c r="AI11" t="str">
-        <v>FLYING OVER ELAFONISI (4K UHD) – Soothing Music Along With Beautiful Nature Video -4K Video ULTRA HD</v>
+        <v>Seagrapes project documentary by WWF SI</v>
       </c>
       <c r="AJ11" t="str">
         <v>4K</v>
@@ -2335,7 +2335,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube</v>
       </c>
       <c r="AM11" t="str">
-        <v>2026-08-01T13:51:43.933Z</v>
+        <v>2026-08-01T16:54:42.980Z</v>
       </c>
       <c r="AN11">
         <v>0.99</v>
@@ -2383,10 +2383,10 @@
         <v>1090</v>
       </c>
       <c r="BC11">
-        <v>4450</v>
+        <v>5472</v>
       </c>
       <c r="BD11">
-        <v>3312</v>
+        <v>3648</v>
       </c>
       <c r="BE11" t="str">
         <v>4K</v>
@@ -2490,22 +2490,22 @@
         <v/>
       </c>
       <c r="AD12" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/f/f0/Nymphaea_lotus_1.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/0/05/Australian_Nymphaea_species_or_hybrid.jpg</v>
       </c>
       <c r="AE12" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Nymphaea_lotus_1.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Australian_Nymphaea_species_or_hybrid.jpg</v>
       </c>
       <c r="AF12" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG12" t="str">
-        <v>https://www.youtube.com/watch?v=7qJnTt5ScL4</v>
+        <v>https://www.youtube.com/watch?v=-yeodYApPYk</v>
       </c>
       <c r="AH12" t="str">
-        <v>7qJnTt5ScL4</v>
+        <v>-yeodYApPYk</v>
       </c>
       <c r="AI12" t="str">
-        <v>Water Lilies in lake | 4K Video | Nature &amp; Relax Healing Music | Detailed Description</v>
+        <v>Blue Lily Flower Power: The Sacred Medicine? | Real Stories Full-Length Documentary</v>
       </c>
       <c r="AJ12" t="str">
         <v>4K</v>
@@ -2517,7 +2517,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM12" t="str">
-        <v>2026-08-01T15:17:49.207Z</v>
+        <v>2026-08-01T16:54:47.516Z</v>
       </c>
       <c r="AN12">
         <v>0.97</v>
@@ -2565,16 +2565,16 @@
         <v>1992</v>
       </c>
       <c r="BC12">
-        <v>388</v>
+        <v>2879</v>
       </c>
       <c r="BD12">
-        <v>325</v>
+        <v>3840</v>
       </c>
       <c r="BE12" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF12" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG12" t="str">
         <v>rights-free</v>
@@ -2672,22 +2672,22 @@
         <v/>
       </c>
       <c r="AD13" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/2/24/Cinnamomum_verum_-_K%C3%B6hler%E2%80%93s_Medizinal-Pflanzen-182.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/b/bd/Cinnamon_bark.jpg</v>
       </c>
       <c r="AE13" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Cinnamomum_verum1.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Cinnamon_bark.jpg</v>
       </c>
       <c r="AF13" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG13" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=tykqe1sUGdg</v>
       </c>
       <c r="AH13" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>tykqe1sUGdg</v>
       </c>
       <c r="AI13" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>Documentary Film 📽️🎥 making about cinnamon #srilanka #travelandtourism #nature #cinnamon #spicy 🇱🇰🦚🙏</v>
       </c>
       <c r="AJ13" t="str">
         <v>4K</v>
@@ -2699,7 +2699,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM13" t="str">
-        <v>2026-08-01T15:17:51.221Z</v>
+        <v>2026-08-01T16:54:51.723Z</v>
       </c>
       <c r="AN13">
         <v>0.99</v>
@@ -2747,16 +2747,16 @@
         <v>2004</v>
       </c>
       <c r="BC13">
-        <v>500</v>
+        <v>4326</v>
       </c>
       <c r="BD13">
-        <v>323</v>
+        <v>2153</v>
       </c>
       <c r="BE13" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF13" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG13" t="str">
         <v>rights-free</v>
@@ -2857,19 +2857,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/8/85/%E1%80%84%E1%80%9B%E1%80%AF%E1%80%90%E1%80%BA%E1%80%80%E1%80%B1%E1%80%AC%E1%80%84%E1%80%BA%E1%80%B8.jpg</v>
       </c>
       <c r="AE14" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Piper_nigrum_-_K%C3%B6hler%E2%80%93s_Medizinal-Pflanzen-107.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:%E1%80%84%E1%80%9B%E1%80%AF%E1%80%90%E1%80%BA%E1%80%80%E1%80%B1%E1%80%AC%E1%80%84%E1%80%BA%E1%80%B8.jpg</v>
       </c>
       <c r="AF14" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG14" t="str">
-        <v>https://www.youtube.com/watch?v=LkZl4HcVVB8</v>
+        <v>https://www.youtube.com/watch?v=W-K_OuzeUSo</v>
       </c>
       <c r="AH14" t="str">
-        <v>LkZl4HcVVB8</v>
+        <v>W-K_OuzeUSo</v>
       </c>
       <c r="AI14" t="str">
-        <v>Jungle Animals in 4K UHD 🌿 | Amazing Wildlife Discovery | 60FPS Ultra HD Nature Documentary</v>
+        <v>How Vietnamese Farmers Harvest Tons of Black Pepper | Farming Documentary</v>
       </c>
       <c r="AJ14" t="str">
         <v>4K</v>
@@ -2881,7 +2881,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM14" t="str">
-        <v>2026-08-01T15:17:53.540Z</v>
+        <v>2026-08-01T16:54:57.332Z</v>
       </c>
       <c r="AN14">
         <v>0.97</v>
@@ -2929,16 +2929,16 @@
         <v>2127</v>
       </c>
       <c r="BC14">
-        <v>466</v>
+        <v>4000</v>
       </c>
       <c r="BD14">
-        <v>595</v>
+        <v>2992</v>
       </c>
       <c r="BE14" t="str">
         <v>4K</v>
       </c>
       <c r="BF14" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG14" t="str">
         <v>rights-free</v>
@@ -3045,13 +3045,13 @@
         <v>Public Domain</v>
       </c>
       <c r="AG15" t="str">
-        <v>https://www.youtube.com/watch?v=mTE1cJWOClQ</v>
+        <v>https://www.youtube.com/watch?v=5K1_KCFudYM</v>
       </c>
       <c r="AH15" t="str">
-        <v>mTE1cJWOClQ</v>
+        <v>5K1_KCFudYM</v>
       </c>
       <c r="AI15" t="str">
-        <v>FLYING OVER ELAFONISI (4K UHD) – Soothing Music Along With Beautiful Nature Video -4K Video ULTRA HD</v>
+        <v>Hornwort (Ceratophyllum demersum) Hardy Plant for Beginners/Breeding Livebearers</v>
       </c>
       <c r="AJ15" t="str">
         <v>4K</v>
@@ -3063,7 +3063,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM15" t="str">
-        <v>2026-08-01T15:17:55.465Z</v>
+        <v>2026-08-01T16:55:01.553Z</v>
       </c>
       <c r="AN15">
         <v>0.97</v>
@@ -3218,22 +3218,22 @@
         <v/>
       </c>
       <c r="AD16" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/6/66/Bley%2C_Botanisches_Bilderbuch_32.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/7/72/Acorus_calamus_SYNTYPE.jpg</v>
       </c>
       <c r="AE16" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Acorus_calamus_rhizomes.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Acorus_calamus_SYNTYPE.jpg</v>
       </c>
       <c r="AF16" t="str">
         <v>CC0</v>
       </c>
       <c r="AG16" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=hD4xkipVgSk</v>
       </c>
       <c r="AH16" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>hD4xkipVgSk</v>
       </c>
       <c r="AI16" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>Acorus Calamus and Acorus Gramineus</v>
       </c>
       <c r="AJ16" t="str">
         <v>4K</v>
@@ -3245,7 +3245,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM16" t="str">
-        <v>2026-08-01T15:17:58.097Z</v>
+        <v>2026-08-01T16:55:05.471Z</v>
       </c>
       <c r="AN16">
         <v>0.99</v>
@@ -3293,10 +3293,10 @@
         <v>2151</v>
       </c>
       <c r="BC16">
-        <v>1540</v>
+        <v>500</v>
       </c>
       <c r="BD16">
-        <v>1155</v>
+        <v>775</v>
       </c>
       <c r="BE16" t="str">
         <v>HD</v>
@@ -3409,13 +3409,13 @@
         <v>Public Domain</v>
       </c>
       <c r="AG17" t="str">
-        <v>https://www.youtube.com/watch?v=qSm93-hhZGg</v>
+        <v>https://www.youtube.com/watch?v=l96_95qbYmM</v>
       </c>
       <c r="AH17" t="str">
-        <v>qSm93-hhZGg</v>
+        <v>l96_95qbYmM</v>
       </c>
       <c r="AI17" t="str">
-        <v>Daintree Rainforest Documentary in 4K | Australia Nature | Queensland | Original Documentary</v>
+        <v>Eat The Weeds: Episode 99: Commelinas, Dayflowers</v>
       </c>
       <c r="AJ17" t="str">
         <v>4K</v>
@@ -3427,7 +3427,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM17" t="str">
-        <v>2026-08-01T15:18:00.056Z</v>
+        <v>2026-08-01T16:55:09.450Z</v>
       </c>
       <c r="AN17">
         <v>0.97</v>
@@ -3585,19 +3585,19 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/381096830/original.jpg</v>
       </c>
       <c r="AE18" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:EB1911_-_Lily_-_Madonna_or_White_Lily_(Lilium_candidum).jpg</v>
+        <v>https://www.inaturalist.org/photos/381096830</v>
       </c>
       <c r="AF18" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG18" t="str">
-        <v>https://www.youtube.com/watch?v=RwDGtbouoY0</v>
+        <v>https://www.youtube.com/watch?v=fNnUnWaawWo</v>
       </c>
       <c r="AH18" t="str">
-        <v>RwDGtbouoY0</v>
+        <v>fNnUnWaawWo</v>
       </c>
       <c r="AI18" t="str">
-        <v>The Most Beautiful Animals on Earth Relaxing 4K Nature Documentary</v>
+        <v>All About Lilies | The Amazing World of the Lily Flower Plant Facts Educational Garden Nature Video</v>
       </c>
       <c r="AJ18" t="str">
         <v>4K</v>
@@ -3609,7 +3609,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM18" t="str">
-        <v>2026-08-01T15:02:06.964Z</v>
+        <v>2026-08-01T16:55:13.341Z</v>
       </c>
       <c r="AN18">
         <v>0.98</v>
@@ -3657,16 +3657,16 @@
         <v>2187</v>
       </c>
       <c r="BC18">
-        <v>292</v>
+        <v>1542</v>
       </c>
       <c r="BD18">
-        <v>451</v>
+        <v>2048</v>
       </c>
       <c r="BE18" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF18" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG18" t="str">
         <v>rights-free</v>
@@ -3764,22 +3764,22 @@
         <v/>
       </c>
       <c r="AD19" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/5/5d/Pandanus_tectorius_aerial_roots_trained_as_an_arch_at_Guam_Zoo%2C_Tumon.jpg</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/507730839/original.jpg</v>
       </c>
       <c r="AE19" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Pandanus_tectorius_aerial_roots_trained_as_an_arch_at_Guam_Zoo,_Tumon.jpg</v>
+        <v>https://www.inaturalist.org/photos/507730839</v>
       </c>
       <c r="AF19" t="str">
         <v>CC0</v>
       </c>
       <c r="AG19" t="str">
-        <v>https://www.youtube.com/watch?v=qSm93-hhZGg</v>
+        <v>https://www.youtube.com/watch?v=iqY4KcOPMJs</v>
       </c>
       <c r="AH19" t="str">
-        <v>qSm93-hhZGg</v>
+        <v>iqY4KcOPMJs</v>
       </c>
       <c r="AI19" t="str">
-        <v>Daintree Rainforest Documentary in 4K | Australia Nature | Queensland | Original Documentary</v>
+        <v>Screw Pine Mini Documentary</v>
       </c>
       <c r="AJ19" t="str">
         <v>4K</v>
@@ -3791,7 +3791,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM19" t="str">
-        <v>2026-08-01T15:18:04.047Z</v>
+        <v>2026-08-01T16:55:17.250Z</v>
       </c>
       <c r="AN19">
         <v>0.97</v>
@@ -3839,16 +3839,16 @@
         <v>2193</v>
       </c>
       <c r="BC19">
-        <v>605</v>
+        <v>1536</v>
       </c>
       <c r="BD19">
-        <v>1280</v>
+        <v>2048</v>
       </c>
       <c r="BE19" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF19" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG19" t="str">
         <v>rights-free</v>
@@ -3949,19 +3949,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/2/28/Ilex_aquifolium_163975455.jpg</v>
       </c>
       <c r="AE20" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Ilex_aquifolium_L._%22Madame_Briot%22_JdP.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Ilex_aquifolium_163975455.jpg</v>
       </c>
       <c r="AF20" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG20" t="str">
-        <v>https://www.youtube.com/watch?v=geOHNKd5jGo</v>
+        <v>https://www.youtube.com/watch?v=kLqRI_CIyoc</v>
       </c>
       <c r="AH20" t="str">
-        <v>geOHNKd5jGo</v>
+        <v>kLqRI_CIyoc</v>
       </c>
       <c r="AI20" t="str">
-        <v>WILD ANTARCTICA: The Icy World of Our Planet Documentary | 4K Ultra HD</v>
+        <v>Nature Insights - A Male Holly (Ilex aquifolium) Tree</v>
       </c>
       <c r="AJ20" t="str">
         <v>4K</v>
@@ -3973,7 +3973,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM20" t="str">
-        <v>2026-08-01T15:18:06.514Z</v>
+        <v>2026-08-01T16:55:21.005Z</v>
       </c>
       <c r="AN20">
         <v>0.97</v>
@@ -4021,16 +4021,16 @@
         <v>2229</v>
       </c>
       <c r="BC20">
-        <v>4592</v>
+        <v>1536</v>
       </c>
       <c r="BD20">
-        <v>3056</v>
+        <v>2048</v>
       </c>
       <c r="BE20" t="str">
-        <v>4K</v>
+        <v>Full HD</v>
       </c>
       <c r="BF20" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG20" t="str">
         <v>rights-free</v>
@@ -4131,19 +4131,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/f/fb/Cosmos_bipinnatus_%28flowers%29_01.jpg</v>
       </c>
       <c r="AE21" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Cosmos_bipinnatus_in_Jardin_universitaire_Roger-Van_den_Hende,_Quebec_city,_Quebec,_Canada.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Cosmos_bipinnatus_(flowers)_01.jpg</v>
       </c>
       <c r="AF21" t="str">
         <v>CC0</v>
       </c>
       <c r="AG21" t="str">
-        <v>https://www.youtube.com/watch?v=cdg4pmLY5Yw</v>
+        <v>https://www.youtube.com/watch?v=bxyjG59bBXE</v>
       </c>
       <c r="AH21" t="str">
-        <v>cdg4pmLY5Yw</v>
+        <v>bxyjG59bBXE</v>
       </c>
       <c r="AI21" t="str">
-        <v>THE COSMOS AND BEYOND 2 : A Cosmic Voyage in 4K UHD + Ambient Space Music by Nature Relaxation™</v>
+        <v>Beautiful autumn cosmos flowers | Nature Scenery Documentary 4K</v>
       </c>
       <c r="AJ21" t="str">
         <v>4K</v>
@@ -4155,7 +4155,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM21" t="str">
-        <v>2026-08-01T15:18:08.967Z</v>
+        <v>2026-08-01T16:55:25.002Z</v>
       </c>
       <c r="AN21">
         <v>0.99</v>
@@ -4203,10 +4203,10 @@
         <v>2235</v>
       </c>
       <c r="BC21">
-        <v>4107</v>
+        <v>4000</v>
       </c>
       <c r="BD21">
-        <v>3631</v>
+        <v>3000</v>
       </c>
       <c r="BE21" t="str">
         <v>4K</v>
@@ -4319,13 +4319,13 @@
         <v>Public Domain</v>
       </c>
       <c r="AG22" t="str">
-        <v>https://www.youtube.com/watch?v=lDEv7jMaiuI</v>
+        <v>https://www.youtube.com/watch?v=QgRpsTaql80</v>
       </c>
       <c r="AH22" t="str">
-        <v>lDEv7jMaiuI</v>
+        <v>QgRpsTaql80</v>
       </c>
       <c r="AI22" t="str">
-        <v>The Amazon Forest in Gentle Motion | Calm Wildlife Documentary in 4K Ultra HD</v>
+        <v>Chrysanthemum morifolium</v>
       </c>
       <c r="AJ22" t="str">
         <v>4K</v>
@@ -4337,7 +4337,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM22" t="str">
-        <v>2026-08-01T15:18:11.297Z</v>
+        <v>2026-08-01T16:55:28.567Z</v>
       </c>
       <c r="AN22">
         <v>0.97</v>
@@ -4492,22 +4492,22 @@
         <v/>
       </c>
       <c r="AD23" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/b/b4/Brassica_oleracea_-_Royal_Botanical_Garden%2C_Madrid.JPG</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/e/e7/Romanescu_Microscopy_02.jpg</v>
       </c>
       <c r="AE23" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Brassica_oleracea_2011_G1.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Romanescu_Microscopy_02.jpg</v>
       </c>
       <c r="AF23" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG23" t="str">
-        <v>https://www.youtube.com/watch?v=xx3kjaERt1M</v>
+        <v>https://www.youtube.com/watch?v=uDdJr1-7tJs</v>
       </c>
       <c r="AH23" t="str">
-        <v>xx3kjaERt1M</v>
+        <v>uDdJr1-7tJs</v>
       </c>
       <c r="AI23" t="str">
-        <v>Secrets of the Outback | Australia's Harshest Wilderness | Full Documentary 4K</v>
+        <v>One Plant. Eight Vegetables. Thousands of Years of Humans Being Picky (Brassica oleracea)</v>
       </c>
       <c r="AJ23" t="str">
         <v>4K</v>
@@ -4519,7 +4519,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM23" t="str">
-        <v>2026-08-01T15:18:13.806Z</v>
+        <v>2026-08-01T16:55:33.534Z</v>
       </c>
       <c r="AN23">
         <v>0.98</v>
@@ -4567,16 +4567,16 @@
         <v>2266</v>
       </c>
       <c r="BC23">
-        <v>4020</v>
+        <v>4000</v>
       </c>
       <c r="BD23">
-        <v>3450</v>
+        <v>3000</v>
       </c>
       <c r="BE23" t="str">
         <v>4K</v>
       </c>
       <c r="BF23" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG23" t="str">
         <v>rights-free</v>
@@ -4683,13 +4683,13 @@
         <v>CC0</v>
       </c>
       <c r="AG24" t="str">
-        <v>https://www.youtube.com/watch?v=qqsrizdiaus</v>
+        <v>https://www.youtube.com/watch?v=TgJs9a6L_TI</v>
       </c>
       <c r="AH24" t="str">
-        <v>qqsrizdiaus</v>
+        <v>TgJs9a6L_TI</v>
       </c>
       <c r="AI24" t="str">
-        <v>🌸 Beautiful Flowers in 4K | Where Nature Blooms Without End</v>
+        <v>Creeping Bellflower, identification of the Wisconsin Invasive Species Campanula rapunculoides</v>
       </c>
       <c r="AJ24" t="str">
         <v>4K</v>
@@ -4701,7 +4701,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM24" t="str">
-        <v>2026-08-01T15:18:16.132Z</v>
+        <v>2026-08-01T16:55:38.241Z</v>
       </c>
       <c r="AN24">
         <v>0.99</v>
@@ -4859,19 +4859,19 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/6561004/original.jpeg</v>
       </c>
       <c r="AE25" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Cornus_florida_-_line_drawing_of_flowering_dogwood_from_USDA_Plants_Database.jpg</v>
+        <v>https://www.inaturalist.org/photos/6561004</v>
       </c>
       <c r="AF25" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG25" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=ptHYhDlnMD8</v>
       </c>
       <c r="AH25" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>ptHYhDlnMD8</v>
       </c>
       <c r="AI25" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>5 Favorite Flowering Dogwood Trees | NatureHills.com</v>
       </c>
       <c r="AJ25" t="str">
         <v>4K</v>
@@ -4883,7 +4883,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM25" t="str">
-        <v>2026-08-01T15:02:19.720Z</v>
+        <v>2026-08-01T16:55:42.895Z</v>
       </c>
       <c r="AN25">
         <v>0.98</v>
@@ -4931,16 +4931,16 @@
         <v>2315</v>
       </c>
       <c r="BC25">
-        <v>600</v>
+        <v>453</v>
       </c>
       <c r="BD25">
-        <v>900</v>
+        <v>647</v>
       </c>
       <c r="BE25" t="str">
         <v/>
       </c>
       <c r="BF25" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG25" t="str">
         <v>rights-free</v>
@@ -5041,7 +5041,7 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/0/0c/Federal_Register_1975-07-01-_Vol_40_Iss_127_%28IA_sim_federal-register-find_1975-07-01_40_127_3%29.pdf</v>
       </c>
       <c r="AE26" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Zoe%3Fa_biological_journal._(IA_mobot31753003412910).pdf</v>
+        <v>https://commons.wikimedia.org/wiki/File:Federal_Register_1975-07-01-_Vol_40_Iss_127_(IA_sim_federal-register-find_1975-07-01_40_127_3).pdf</v>
       </c>
       <c r="AF26" t="str">
         <v>Public Domain</v>
@@ -5065,7 +5065,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM26" t="str">
-        <v>2026-08-01T15:18:21.165Z</v>
+        <v>2026-08-01T16:55:46.249Z</v>
       </c>
       <c r="AN26">
         <v>0.99</v>
@@ -5113,13 +5113,13 @@
         <v>2321</v>
       </c>
       <c r="BC26">
-        <v>4222</v>
+        <v>1220</v>
       </c>
       <c r="BD26">
-        <v>6637</v>
+        <v>1700</v>
       </c>
       <c r="BE26" t="str">
-        <v>4K</v>
+        <v>HD</v>
       </c>
       <c r="BF26" t="str">
         <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
@@ -5223,22 +5223,22 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/646898160/original.jpg</v>
       </c>
       <c r="AE27" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Dillenia_indica_fruit.jpg</v>
+        <v>https://www.inaturalist.org/photos/646898160</v>
       </c>
       <c r="AF27" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG27" t="str">
-        <v>https://www.youtube.com/watch?v=qoZvjM3Anek</v>
+        <v>https://www.youtube.com/watch?v=-AshqUhPotU</v>
       </c>
       <c r="AH27" t="str">
-        <v>qoZvjM3Anek</v>
+        <v>-AshqUhPotU</v>
       </c>
       <c r="AI27" t="str">
-        <v>Namibia's Living Desert: A Story of Adaptation and Survival | 4K UHD Documentary</v>
+        <v>life of Dillenia indica . life full hd</v>
       </c>
       <c r="AJ27" t="str">
-        <v>4K</v>
+        <v>HD</v>
       </c>
       <c r="AK27" t="str">
         <v>https://www.gbif.org/species/5383898</v>
@@ -5247,7 +5247,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM27" t="str">
-        <v>2026-08-01T15:02:23.545Z</v>
+        <v>2026-08-01T16:55:50.993Z</v>
       </c>
       <c r="AN27">
         <v>0.97</v>
@@ -5295,16 +5295,16 @@
         <v>2333</v>
       </c>
       <c r="BC27">
-        <v>1024</v>
+        <v>1536</v>
       </c>
       <c r="BD27">
-        <v>768</v>
+        <v>2048</v>
       </c>
       <c r="BE27" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF27" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG27" t="str">
         <v>rights-free</v>
@@ -5402,22 +5402,22 @@
         <v/>
       </c>
       <c r="AD28" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/f/fc/Soybeanvarieties.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/d/d9/Soy_field_in_Granville_County.jpg</v>
       </c>
       <c r="AE28" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Glycine_max_Taub131a.png</v>
+        <v>https://commons.wikimedia.org/wiki/File:Soy_field_in_Granville_County.jpg</v>
       </c>
       <c r="AF28" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG28" t="str">
-        <v>https://www.youtube.com/watch?v=ZnZBRZYVRNU</v>
+        <v>https://www.youtube.com/watch?v=QuEXKwQzUOQ</v>
       </c>
       <c r="AH28" t="str">
-        <v>ZnZBRZYVRNU</v>
+        <v>QuEXKwQzUOQ</v>
       </c>
       <c r="AI28" t="str">
-        <v>4K Amazing Animals in the Wild Wildlife Documentary 4K Ultra HD Animal World HD</v>
+        <v>125 Billion Pounds Of Soybean Harvested By American Farmers This Way | Farming Documentary</v>
       </c>
       <c r="AJ28" t="str">
         <v>4K</v>
@@ -5429,7 +5429,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM28" t="str">
-        <v>2026-08-01T15:18:25.756Z</v>
+        <v>2026-08-01T16:55:55.492Z</v>
       </c>
       <c r="AN28">
         <v>0.99</v>
@@ -5477,16 +5477,16 @@
         <v>2357</v>
       </c>
       <c r="BC28">
-        <v>940</v>
+        <v>2340</v>
       </c>
       <c r="BD28">
-        <v>1185</v>
+        <v>2512</v>
       </c>
       <c r="BE28" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF28" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG28" t="str">
         <v>rights-free</v>
@@ -5587,19 +5587,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/0/05/Dettaglio_-_Cupuliferae_Quercus_robur_Lin._-_Erbario_Frizzi_Perugia_n._1518.jpg</v>
       </c>
       <c r="AE29" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:New_oak_leaves_with_female_flowers.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Dettaglio_-_Cupuliferae_Quercus_robur_Lin._-_Erbario_Frizzi_Perugia_n._1518.jpg</v>
       </c>
       <c r="AF29" t="str">
-        <v>CC0</v>
+        <v>Public Domain</v>
       </c>
       <c r="AG29" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=QpzZxdrtJl0</v>
       </c>
       <c r="AH29" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>QpzZxdrtJl0</v>
       </c>
       <c r="AI29" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>Learn UK Trees - English Oak (Quercus robur)</v>
       </c>
       <c r="AJ29" t="str">
         <v>4K</v>
@@ -5611,7 +5611,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM29" t="str">
-        <v>2026-08-01T15:18:28.400Z</v>
+        <v>2026-08-01T16:55:59.685Z</v>
       </c>
       <c r="AN29">
         <v>0.97</v>
@@ -5659,16 +5659,16 @@
         <v>2363</v>
       </c>
       <c r="BC29">
-        <v>3720</v>
+        <v>1705</v>
       </c>
       <c r="BD29">
-        <v>2790</v>
+        <v>2656</v>
       </c>
       <c r="BE29" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF29" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
       </c>
       <c r="BG29" t="str">
         <v>rights-free</v>
@@ -5775,13 +5775,13 @@
         <v>CC0</v>
       </c>
       <c r="AG30" t="str">
-        <v>https://www.youtube.com/watch?v=PlRSanFP6nw</v>
+        <v>https://www.youtube.com/watch?v=jKzVqtIMs7A</v>
       </c>
       <c r="AH30" t="str">
-        <v>PlRSanFP6nw</v>
+        <v>jKzVqtIMs7A</v>
       </c>
       <c r="AI30" t="str">
-        <v>Australia Nature Documentary 4K | K’gari (Fraser Island) | Wildlife and Natural History</v>
+        <v>Garrya elliptica, Garryaceae</v>
       </c>
       <c r="AJ30" t="str">
         <v>4K</v>
@@ -5793,7 +5793,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM30" t="str">
-        <v>2026-08-01T15:18:30.769Z</v>
+        <v>2026-08-01T16:56:03.743Z</v>
       </c>
       <c r="AN30">
         <v>0.97</v>
@@ -6139,13 +6139,13 @@
         <v>Public Domain</v>
       </c>
       <c r="AG32" t="str">
-        <v>https://www.youtube.com/watch?v=Ygk-odokFUs</v>
+        <v>https://www.youtube.com/watch?v=8M29t0GcNqI</v>
       </c>
       <c r="AH32" t="str">
-        <v>Ygk-odokFUs</v>
+        <v>8M29t0GcNqI</v>
       </c>
       <c r="AI32" t="str">
-        <v>Catching Giant Millipedes in Rubber Tree Farm 🐛 | Amazing Night Hunt in the Wild (4K)</v>
+        <v>Hidden Forest: The Animals You Never Knew Lived in Trees | FULL DOCUMENTARY | Wildest Survival</v>
       </c>
       <c r="AJ32" t="str">
         <v>4K</v>
@@ -6157,7 +6157,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM32" t="str">
-        <v>2026-08-01T15:18:35.166Z</v>
+        <v>2026-08-01T16:56:11.421Z</v>
       </c>
       <c r="AN32">
         <v>0.99</v>
@@ -6312,22 +6312,22 @@
         <v/>
       </c>
       <c r="AD33" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/0/0a/Ochna_integerrima_2_-_Chiang_Mai.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/6/64/Hoa_mai.jpg</v>
       </c>
       <c r="AE33" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Ochna_integerrima_2_-_Chiang_Mai.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Hoa_mai.jpg</v>
       </c>
       <c r="AF33" t="str">
-        <v>CC0</v>
+        <v>Public Domain</v>
       </c>
       <c r="AG33" t="str">
-        <v>https://www.youtube.com/watch?v=dF1X13Oo0pg</v>
+        <v>https://www.youtube.com/watch?v=NpQ1X4J3rzM</v>
       </c>
       <c r="AH33" t="str">
-        <v>dF1X13Oo0pg</v>
+        <v>NpQ1X4J3rzM</v>
       </c>
       <c r="AI33" t="str">
-        <v>10 Hours of Epic 4K Wildlife Documentary: Crocodiles Buffaloes &amp; Nature’s Greatest Battles #wildlife</v>
+        <v>WILD YELLOWSTONE | Ruthless Predators and Majestic Wilderness | Nature animal documentary</v>
       </c>
       <c r="AJ33" t="str">
         <v>4K</v>
@@ -6339,7 +6339,7 @@
         <v>gbif | wikimedia | youtube</v>
       </c>
       <c r="AM33" t="str">
-        <v>2026-08-01T13:53:26.845Z</v>
+        <v>2026-08-01T16:56:14.987Z</v>
       </c>
       <c r="AN33">
         <v>0.99</v>
@@ -6387,16 +6387,16 @@
         <v>2417</v>
       </c>
       <c r="BC33">
-        <v>3060</v>
+        <v>1407</v>
       </c>
       <c r="BD33">
-        <v>4080</v>
+        <v>2769</v>
       </c>
       <c r="BE33" t="str">
-        <v>4K</v>
+        <v>Full HD</v>
       </c>
       <c r="BF33" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
       </c>
       <c r="BG33" t="str">
         <v>rights-free</v>
@@ -6494,22 +6494,22 @@
         <v/>
       </c>
       <c r="AD34" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/c/c3/Eucalyptus_globulus_-_K%C3%B6hler%E2%80%93s_Medizinal-Pflanzen-147.jpg</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/348028899/original.jpeg</v>
       </c>
       <c r="AE34" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Eucalyptus_globulus_Labillardi%C3%A8re.jpg</v>
+        <v>https://www.inaturalist.org/photos/348028899</v>
       </c>
       <c r="AF34" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG34" t="str">
-        <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
+        <v>https://www.youtube.com/watch?v=ugX-ubVNxZM</v>
       </c>
       <c r="AH34" t="str">
-        <v>dSsubsLx2ZA</v>
+        <v>ugX-ubVNxZM</v>
       </c>
       <c r="AI34" t="str">
-        <v>The Incredible Scottish Highlands (4K Documentary) | Our World</v>
+        <v>Koala Country: Survival in Australia's Changing Eucalyptus Forest | Wild Tales | Documentary</v>
       </c>
       <c r="AJ34" t="str">
         <v>4K</v>
@@ -6521,7 +6521,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM34" t="str">
-        <v>2026-08-01T15:18:39.633Z</v>
+        <v>2026-08-01T16:56:19.116Z</v>
       </c>
       <c r="AN34">
         <v>0.99</v>
@@ -6569,16 +6569,16 @@
         <v>2435</v>
       </c>
       <c r="BC34">
-        <v>864</v>
+        <v>1152</v>
       </c>
       <c r="BD34">
-        <v>1500</v>
+        <v>2048</v>
       </c>
       <c r="BE34" t="str">
-        <v>HD</v>
+        <v>Full HD</v>
       </c>
       <c r="BF34" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG34" t="str">
         <v>rights-free</v>
@@ -6676,22 +6676,22 @@
         <v/>
       </c>
       <c r="AD35" t="str">
-        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/327107588/original.jpeg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/4/44/Oxalis_corniculata%2C_2020-09-09%2C_Beechview%2C_01.jpg</v>
       </c>
       <c r="AE35" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Oxalis_corniculata,_2020-09-09,_Beechview,_02.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Oxalis_corniculata,_2020-09-09,_Beechview,_01.jpg</v>
       </c>
       <c r="AF35" t="str">
         <v>CC0</v>
       </c>
       <c r="AG35" t="str">
-        <v>https://www.youtube.com/watch?v=8_lLAEEvty4</v>
+        <v>https://www.youtube.com/watch?v=KIZQYEf1prM</v>
       </c>
       <c r="AH35" t="str">
-        <v>8_lLAEEvty4</v>
+        <v>KIZQYEf1prM</v>
       </c>
       <c r="AI35" t="str">
-        <v>The Most Extraordinary Birds on Earth | 4K Wildlife Documentary</v>
+        <v>Day 10: Spring Nature Connection/ Foraging- Meet Wood Sorrel (Oxalis acetosella)</v>
       </c>
       <c r="AJ35" t="str">
         <v>4K</v>
@@ -6703,7 +6703,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM35" t="str">
-        <v>2026-08-01T15:02:38.503Z</v>
+        <v>2026-08-01T16:56:23.025Z</v>
       </c>
       <c r="AN35">
         <v>0.99</v>
@@ -6751,10 +6751,10 @@
         <v>2441</v>
       </c>
       <c r="BC35">
-        <v>2448</v>
+        <v>2188</v>
       </c>
       <c r="BD35">
-        <v>3264</v>
+        <v>2188</v>
       </c>
       <c r="BE35" t="str">
         <v>Full HD</v>
@@ -7231,13 +7231,13 @@
         <v>CC0</v>
       </c>
       <c r="AG38" t="str">
-        <v>https://www.youtube.com/watch?v=KW8vZY9pW7k</v>
+        <v>https://www.youtube.com/watch?v=yXbD1mq969E</v>
       </c>
       <c r="AH38" t="str">
-        <v>KW8vZY9pW7k</v>
+        <v>yXbD1mq969E</v>
       </c>
       <c r="AI38" t="str">
-        <v>Alaska’s Untamed Beauty 4K: Untouched Wilderness &amp; Incredible Wildlife</v>
+        <v>Macadamia integrifolia 4K, 120 years old</v>
       </c>
       <c r="AJ38" t="str">
         <v>4K</v>
@@ -7249,7 +7249,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM38" t="str">
-        <v>2026-08-01T15:18:47.259Z</v>
+        <v>2026-08-01T16:56:32.407Z</v>
       </c>
       <c r="AN38">
         <v>0.99</v>
@@ -7407,19 +7407,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/8/8b/Zentralbibliothek_Z%C3%BCrich_-_Pfirsichspalier_gr%C3%B6sser_-_991124120369705501.jpg</v>
       </c>
       <c r="AE39" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Autumn_Red_peaches.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Zentralbibliothek_Z%C3%BCrich_-_Pfirsichspalier_gr%C3%B6sser_-_991124120369705501.jpg</v>
       </c>
       <c r="AF39" t="str">
         <v>Public Domain</v>
       </c>
       <c r="AG39" t="str">
-        <v>https://www.youtube.com/watch?v=CJAQQa_FlLs</v>
+        <v>https://www.youtube.com/watch?v=2VLCac-2wkA</v>
       </c>
       <c r="AH39" t="str">
-        <v>CJAQQa_FlLs</v>
+        <v>2VLCac-2wkA</v>
       </c>
       <c r="AI39" t="str">
-        <v>Dreamy peach blossoms scenery in Niyodogawa town | Nature Scenery Documentary 4K</v>
+        <v>Tibet 4K Nyingchi Valley: Peach Blossom Village</v>
       </c>
       <c r="AJ39" t="str">
         <v>4K</v>
@@ -7431,7 +7431,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM39" t="str">
-        <v>2026-08-01T15:18:49.605Z</v>
+        <v>2026-08-01T16:56:37.127Z</v>
       </c>
       <c r="AN39">
         <v>0.97</v>
@@ -7479,13 +7479,13 @@
         <v>2477</v>
       </c>
       <c r="BC39">
-        <v>2784</v>
+        <v>4462</v>
       </c>
       <c r="BD39">
-        <v>1896</v>
+        <v>3920</v>
       </c>
       <c r="BE39" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF39" t="str">
         <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
@@ -7768,22 +7768,22 @@
         <v/>
       </c>
       <c r="AD41" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/c/cf/Zentralbibliothek_Z%C3%BCrich_-_Landgut_Bocken_von_S%C3%BCdwest_-_991154996899705501.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/7/75/Zentralbibliothek_Z%C3%BCrich_-_Ulme_vor_d._Haus_-_991021389379705501.jpg</v>
       </c>
       <c r="AE41" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Small_greenhouse_with_grapevines_escaping.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Zentralbibliothek_Z%C3%BCrich_-_Ulme_vor_d._Haus_-_991021389379705501.jpg</v>
       </c>
       <c r="AF41" t="str">
-        <v>CC0</v>
+        <v>Public Domain</v>
       </c>
       <c r="AG41" t="str">
-        <v>https://www.youtube.com/watch?v=LkZl4HcVVB8</v>
+        <v>https://www.youtube.com/watch?v=I6Xg90Y-IOs</v>
       </c>
       <c r="AH41" t="str">
-        <v>LkZl4HcVVB8</v>
+        <v>I6Xg90Y-IOs</v>
       </c>
       <c r="AI41" t="str">
-        <v>Jungle Animals in 4K UHD 🌿 | Amazing Wildlife Discovery | 60FPS Ultra HD Nature Documentary</v>
+        <v>The Amazing Life Cycle of Grapes 🍇 | From Seed to Grape Vine Time Lapse | AI Nature Documentary 4K</v>
       </c>
       <c r="AJ41" t="str">
         <v>4K</v>
@@ -7795,7 +7795,7 @@
         <v>gbif | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM41" t="str">
-        <v>2026-08-01T15:18:54.161Z</v>
+        <v>2026-08-01T16:56:45.233Z</v>
       </c>
       <c r="AN41">
         <v>0.97</v>
@@ -7843,16 +7843,16 @@
         <v>2513</v>
       </c>
       <c r="BC41">
-        <v>8972</v>
+        <v>4420</v>
       </c>
       <c r="BD41">
-        <v>5645</v>
+        <v>3934</v>
       </c>
       <c r="BE41" t="str">
         <v>4K</v>
       </c>
       <c r="BF41" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
       </c>
       <c r="BG41" t="str">
         <v>rights-free</v>
@@ -8135,10 +8135,10 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/2/2b/%E1%80%94%E1%80%B6%E1%80%94%E1%80%B6%E1%80%95%E1%80%84%E1%80%BA%E1%80%99%E1%80%BD%E1%80%BE%E1%80%B1%E1%80%B8.jpg</v>
       </c>
       <c r="AE43" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Illustration_Coriandrum_sativum0.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:%E1%80%94%E1%80%B6%E1%80%94%E1%80%B6%E1%80%95%E1%80%84%E1%80%BA%E1%80%99%E1%80%BD%E1%80%BE%E1%80%B1%E1%80%B8.jpg</v>
       </c>
       <c r="AF43" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG43" t="str">
         <v>https://www.youtube.com/watch?v=dSsubsLx2ZA</v>
@@ -8159,7 +8159,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM43" t="str">
-        <v>2026-08-01T15:18:58.457Z</v>
+        <v>2026-08-01T16:56:52.766Z</v>
       </c>
       <c r="AN43">
         <v>0.94</v>
@@ -8207,16 +8207,16 @@
         <v>2581</v>
       </c>
       <c r="BC43">
-        <v>1482</v>
+        <v>4000</v>
       </c>
       <c r="BD43">
-        <v>2333</v>
+        <v>2992</v>
       </c>
       <c r="BE43" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF43" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG43" t="str">
         <v>rights-free</v>
@@ -8314,22 +8314,22 @@
         <v/>
       </c>
       <c r="AD44" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/b/b7/Ipomoea_batatoides_Edwards%27s_Bot._Reg._27._36._1841.jpg</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/12388764/original.jpeg</v>
       </c>
       <c r="AE44" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Ipomoea_purpurea_2016_G1.jpg</v>
+        <v>https://www.inaturalist.org/photos/12388764</v>
       </c>
       <c r="AF44" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG44" t="str">
-        <v>https://www.youtube.com/watch?v=7ZhdXgRfxHI</v>
+        <v>https://www.youtube.com/watch?v=59ZwNFmliRw</v>
       </c>
       <c r="AH44" t="str">
-        <v>7ZhdXgRfxHI</v>
+        <v>59ZwNFmliRw</v>
       </c>
       <c r="AI44" t="str">
-        <v>Incredible 4K Nature Scenes Narrated By David Attenborough | BBC Earth</v>
+        <v>India's Silent Green Invasion: The Truth About Ipomoea carnea</v>
       </c>
       <c r="AJ44" t="str">
         <v>4K</v>
@@ -8341,7 +8341,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM44" t="str">
-        <v>2026-08-01T15:19:02.947Z</v>
+        <v>2026-08-01T16:56:57.308Z</v>
       </c>
       <c r="AN44">
         <v>0.92</v>
@@ -8389,16 +8389,16 @@
         <v>2691</v>
       </c>
       <c r="BC44">
-        <v>2700</v>
+        <v>1744</v>
       </c>
       <c r="BD44">
-        <v>3600</v>
+        <v>2048</v>
       </c>
       <c r="BE44" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF44" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG44" t="str">
         <v>rights-free</v>
@@ -8499,10 +8499,10 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/438895859/original.jpeg</v>
       </c>
       <c r="AE45" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Benincasa_illustration.jpg</v>
+        <v>https://www.inaturalist.org/photos/438895859</v>
       </c>
       <c r="AF45" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG45" t="str">
         <v>https://www.youtube.com/watch?v=SIm3nKfJnFE</v>
@@ -8523,7 +8523,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM45" t="str">
-        <v>2026-08-01T15:02:59.405Z</v>
+        <v>2026-08-01T16:57:01.051Z</v>
       </c>
       <c r="AN45">
         <v>0.94</v>
@@ -8571,16 +8571,16 @@
         <v>2701</v>
       </c>
       <c r="BC45">
-        <v>1773</v>
+        <v>2048</v>
       </c>
       <c r="BD45">
-        <v>1080</v>
+        <v>1365</v>
       </c>
       <c r="BE45" t="str">
-        <v>HD</v>
+        <v>Full HD</v>
       </c>
       <c r="BF45" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG45" t="str">
         <v>rights-free</v>
@@ -8681,7 +8681,7 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/400503884/original.jpg</v>
       </c>
       <c r="AE46" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Hopea_parviflora.location_iringole.jpg</v>
+        <v>https://www.inaturalist.org/photos/400503884</v>
       </c>
       <c r="AF46" t="str">
         <v>CC0</v>
@@ -8705,7 +8705,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM46" t="str">
-        <v>2026-08-01T15:03:01.625Z</v>
+        <v>2026-08-01T16:57:04.856Z</v>
       </c>
       <c r="AN46">
         <v>0.92</v>
@@ -8753,16 +8753,16 @@
         <v>2731</v>
       </c>
       <c r="BC46">
-        <v>1000</v>
+        <v>1548</v>
       </c>
       <c r="BD46">
-        <v>665</v>
+        <v>1161</v>
       </c>
       <c r="BE46" t="str">
         <v>HD</v>
       </c>
       <c r="BF46" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG46" t="str">
         <v>rights-free</v>
@@ -8863,10 +8863,10 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/259118694/original.jpeg</v>
       </c>
       <c r="AE47" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Elsholtzia_ciliata-2.jpg</v>
+        <v>https://www.inaturalist.org/photos/259118694</v>
       </c>
       <c r="AF47" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG47" t="str">
         <v>https://www.youtube.com/watch?v=7ZhdXgRfxHI</v>
@@ -8887,7 +8887,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM47" t="str">
-        <v>2026-08-01T15:03:03.503Z</v>
+        <v>2026-08-01T16:57:08.217Z</v>
       </c>
       <c r="AN47">
         <v>0.92</v>
@@ -8935,16 +8935,16 @@
         <v>2781</v>
       </c>
       <c r="BC47">
-        <v>3648</v>
+        <v>1536</v>
       </c>
       <c r="BD47">
-        <v>2736</v>
+        <v>2048</v>
       </c>
       <c r="BE47" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF47" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG47" t="str">
         <v>rights-free</v>
@@ -9042,22 +9042,22 @@
         <v/>
       </c>
       <c r="AD48" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/b/b8/Barringtonia_racemosa_Blanco2.240.png</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/144097536/original.jpeg</v>
       </c>
       <c r="AE48" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Barringtonia_neocaledonica_JdP.jpg</v>
+        <v>https://www.inaturalist.org/photos/144097536</v>
       </c>
       <c r="AF48" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG48" t="str">
-        <v>https://www.youtube.com/watch?v=MDIknO9eqjc</v>
+        <v>https://www.youtube.com/watch?v=qDzF5OSqW0k</v>
       </c>
       <c r="AH48" t="str">
-        <v>MDIknO9eqjc</v>
+        <v>qDzF5OSqW0k</v>
       </c>
       <c r="AI48" t="str">
-        <v>Hidden Lives of Australia's Forests | 4K Nature Documentary</v>
+        <v>Barringtonia asiatica, the fish poison tree</v>
       </c>
       <c r="AJ48" t="str">
         <v>4K</v>
@@ -9069,7 +9069,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM48" t="str">
-        <v>2026-08-01T15:19:12.748Z</v>
+        <v>2026-08-01T16:57:11.963Z</v>
       </c>
       <c r="AN48">
         <v>0.94</v>
@@ -9117,16 +9117,16 @@
         <v>2801</v>
       </c>
       <c r="BC48">
-        <v>4592</v>
+        <v>2048</v>
       </c>
       <c r="BD48">
-        <v>3056</v>
+        <v>1536</v>
       </c>
       <c r="BE48" t="str">
-        <v>4K</v>
+        <v>Full HD</v>
       </c>
       <c r="BF48" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG48" t="str">
         <v>rights-free</v>
@@ -9227,19 +9227,19 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/4/4d/Crape_myrtle_%28Lagerstroemia_sp.%29_Crown_gall_disease_%2849772271993%29.jpg</v>
       </c>
       <c r="AE49" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Lagerstroemia_indica_Blanco1.207.png</v>
+        <v>https://commons.wikimedia.org/wiki/File:Crape_myrtle_(Lagerstroemia_sp.)_Crown_gall_disease_(49772271993).jpg</v>
       </c>
       <c r="AF49" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG49" t="str">
-        <v>https://www.youtube.com/watch?v=O-yyQ6t_B-U</v>
+        <v>https://www.youtube.com/watch?v=U4YJcWhg3-k</v>
       </c>
       <c r="AH49" t="str">
-        <v>O-yyQ6t_B-U</v>
+        <v>U4YJcWhg3-k</v>
       </c>
       <c r="AI49" t="str">
-        <v>Amazon Rainforest 4K Ultra HD 🌿 | Peaceful Jungle Sounds &amp; Exotic Wildlife Documentary</v>
+        <v>Amazing Facts About Lagerstroemia speciosa | PRIDE OF INDIA🤯 #viral #nature #love #explore</v>
       </c>
       <c r="AJ49" t="str">
         <v>4K</v>
@@ -9251,7 +9251,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM49" t="str">
-        <v>2026-08-01T15:19:15.411Z</v>
+        <v>2026-08-01T16:57:17.389Z</v>
       </c>
       <c r="AN49">
         <v>0.94</v>
@@ -9299,16 +9299,16 @@
         <v>2811</v>
       </c>
       <c r="BC49">
-        <v>1417</v>
+        <v>3024</v>
       </c>
       <c r="BD49">
-        <v>2089</v>
+        <v>4032</v>
       </c>
       <c r="BE49" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF49" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG49" t="str">
         <v>rights-free</v>
@@ -9409,10 +9409,10 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/a/a4/Semal_Jaipur.jpg</v>
       </c>
       <c r="AE50" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Bombax_ceiba_Blanco1.226b.png</v>
+        <v>https://commons.wikimedia.org/wiki/File:Semal_Jaipur.jpg</v>
       </c>
       <c r="AF50" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG50" t="str">
         <v>https://www.youtube.com/watch?v=LYGvsTUJFM8</v>
@@ -9433,7 +9433,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM50" t="str">
-        <v>2026-08-01T15:19:17.471Z</v>
+        <v>2026-08-01T16:57:21.938Z</v>
       </c>
       <c r="AN50">
         <v>0.94</v>
@@ -9481,16 +9481,16 @@
         <v>2821</v>
       </c>
       <c r="BC50">
-        <v>1393</v>
+        <v>3060</v>
       </c>
       <c r="BD50">
-        <v>2038</v>
+        <v>4080</v>
       </c>
       <c r="BE50" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF50" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG50" t="str">
         <v>rights-free</v>
@@ -9591,19 +9591,19 @@
         <v>https://inaturalist-open-data.s3.amazonaws.com/photos/129173117/original.jpg</v>
       </c>
       <c r="AE51" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Swietenia_mahagoni_BYN.jpg</v>
+        <v>https://www.inaturalist.org/photos/129173117</v>
       </c>
       <c r="AF51" t="str">
         <v>CC0</v>
       </c>
       <c r="AG51" t="str">
-        <v>https://www.youtube.com/watch?v=7ZhdXgRfxHI</v>
+        <v>https://www.youtube.com/watch?v=pC8Yhw9KWTU</v>
       </c>
       <c r="AH51" t="str">
-        <v>7ZhdXgRfxHI</v>
+        <v>pC8Yhw9KWTU</v>
       </c>
       <c r="AI51" t="str">
-        <v>Incredible 4K Nature Scenes Narrated By David Attenborough | BBC Earth</v>
+        <v>Mahogany Tree (Swietenia macrophylla)</v>
       </c>
       <c r="AJ51" t="str">
         <v>4K</v>
@@ -9615,7 +9615,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM51" t="str">
-        <v>2026-08-01T15:03:10.877Z</v>
+        <v>2026-08-01T16:57:26.231Z</v>
       </c>
       <c r="AN51">
         <v>0.94</v>
@@ -9663,16 +9663,16 @@
         <v>2831</v>
       </c>
       <c r="BC51">
-        <v>2482</v>
+        <v>1536</v>
       </c>
       <c r="BD51">
-        <v>4465</v>
+        <v>2048</v>
       </c>
       <c r="BE51" t="str">
-        <v>4K</v>
+        <v>Full HD</v>
       </c>
       <c r="BF51" t="str">
-        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG51" t="str">
         <v>rights-free</v>
@@ -9770,22 +9770,22 @@
         <v/>
       </c>
       <c r="AD52" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/5/5e/Artocarpus_incisus_Blanco2.267.png</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/b/b9/Artocarpus_chama%2C_Jhapa_District%2C_Mechi%2C_NP_imported_from_iNaturalist_photo_190818146.jpg</v>
       </c>
       <c r="AE52" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Characteres_generum_plantarum_plate_51_Artocarpus.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Artocarpus_chama,_Jhapa_District,_Mechi,_NP_imported_from_iNaturalist_photo_190818146.jpg</v>
       </c>
       <c r="AF52" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG52" t="str">
-        <v>https://www.youtube.com/watch?v=7ZhdXgRfxHI</v>
+        <v>https://www.youtube.com/watch?v=jjugVvQrNC0</v>
       </c>
       <c r="AH52" t="str">
-        <v>7ZhdXgRfxHI</v>
+        <v>jjugVvQrNC0</v>
       </c>
       <c r="AI52" t="str">
-        <v>Incredible 4K Nature Scenes Narrated By David Attenborough | BBC Earth</v>
+        <v>Jackfruit (Artocarpus heterophyllus)</v>
       </c>
       <c r="AJ52" t="str">
         <v>4K</v>
@@ -9797,7 +9797,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM52" t="str">
-        <v>2026-08-01T15:19:22.218Z</v>
+        <v>2026-08-01T16:57:30.207Z</v>
       </c>
       <c r="AN52">
         <v>0.94</v>
@@ -9845,16 +9845,16 @@
         <v>2861</v>
       </c>
       <c r="BC52">
-        <v>477</v>
+        <v>1536</v>
       </c>
       <c r="BD52">
-        <v>753</v>
+        <v>2048</v>
       </c>
       <c r="BE52" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF52" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG52" t="str">
         <v>rights-free</v>
@@ -9952,22 +9952,22 @@
         <v/>
       </c>
       <c r="AD53" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/6/66/06800jfBoats_Bridge_Landscapes_Scenery_Sapang_Bayan_Rivers_Calumpit_Bulacanfvf_12.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/d/d6/Sur_le_pont_du_fleuve_Nyong._03.jpg</v>
       </c>
       <c r="AE53" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:The_Prophet_Musa_(Moses_In_Islam).png</v>
+        <v>https://commons.wikimedia.org/wiki/File:Sur_le_pont_du_fleuve_Nyong._03.jpg</v>
       </c>
       <c r="AF53" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG53" t="str">
-        <v>https://www.youtube.com/watch?v=7ZhdXgRfxHI</v>
+        <v>https://www.youtube.com/watch?v=89s1_wBPQb8</v>
       </c>
       <c r="AH53" t="str">
-        <v>7ZhdXgRfxHI</v>
+        <v>89s1_wBPQb8</v>
       </c>
       <c r="AI53" t="str">
-        <v>Incredible 4K Nature Scenes Narrated By David Attenborough | BBC Earth</v>
+        <v>Mansa Musa - History’s Richest Man Documentary</v>
       </c>
       <c r="AJ53" t="str">
         <v>4K</v>
@@ -9979,7 +9979,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM53" t="str">
-        <v>2026-08-01T15:19:24.841Z</v>
+        <v>2026-08-01T16:57:35.322Z</v>
       </c>
       <c r="AN53">
         <v>0.94</v>
@@ -10027,16 +10027,16 @@
         <v>2871</v>
       </c>
       <c r="BC53">
-        <v>2048</v>
+        <v>3024</v>
       </c>
       <c r="BD53">
-        <v>2048</v>
+        <v>4032</v>
       </c>
       <c r="BE53" t="str">
-        <v>Full HD</v>
+        <v>4K</v>
       </c>
       <c r="BF53" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG53" t="str">
         <v>rights-free</v>
@@ -10143,13 +10143,13 @@
         <v>Public Domain</v>
       </c>
       <c r="AG54" t="str">
-        <v>https://www.youtube.com/watch?v=YUj7yt6iV2w</v>
+        <v>https://www.youtube.com/watch?v=HfnCoVND3Cc</v>
       </c>
       <c r="AH54" t="str">
-        <v>YUj7yt6iV2w</v>
+        <v>HfnCoVND3Cc</v>
       </c>
       <c r="AI54" t="str">
-        <v>4K Nature Documentary Wildlife, Rainforests, Oceans &amp; Mountains in Ultra HD Relaxation Film</v>
+        <v>Fascinating Flora - Ziziphus mucronata buffalo thorn tree with Jarryd</v>
       </c>
       <c r="AJ54" t="str">
         <v>4K</v>
@@ -10161,7 +10161,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM54" t="str">
-        <v>2026-08-01T15:19:27.699Z</v>
+        <v>2026-08-01T16:57:39.725Z</v>
       </c>
       <c r="AN54">
         <v>0.94</v>
@@ -10319,7 +10319,7 @@
         <v>https://upload.wikimedia.org/wikipedia/commons/e/e4/Fruts_banana_oranfe_avocado.jpg</v>
       </c>
       <c r="AE55" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Pears.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Fruts_banana_oranfe_avocado.jpg</v>
       </c>
       <c r="AF55" t="str">
         <v>Public Domain</v>
@@ -10343,7 +10343,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM55" t="str">
-        <v>2026-08-01T15:19:30.460Z</v>
+        <v>2026-08-01T16:57:44.560Z</v>
       </c>
       <c r="AN55">
         <v>0.94</v>
@@ -10391,10 +10391,10 @@
         <v>2941</v>
       </c>
       <c r="BC55">
-        <v>640</v>
+        <v>1920</v>
       </c>
       <c r="BD55">
-        <v>975</v>
+        <v>2560</v>
       </c>
       <c r="BE55" t="str">
         <v>Full HD</v>
@@ -10498,22 +10498,22 @@
         <v/>
       </c>
       <c r="AD56" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/e/e0/Citrus_fruits.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/3/36/Limes_with_halves.jpg</v>
       </c>
       <c r="AE56" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Citrus_fruits.jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Limes_with_halves.jpg</v>
       </c>
       <c r="AF56" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG56" t="str">
-        <v>https://www.youtube.com/watch?v=5X1lECCJ5Mw</v>
+        <v>https://www.youtube.com/watch?v=XkMKJCvJKBk</v>
       </c>
       <c r="AH56" t="str">
-        <v>5X1lECCJ5Mw</v>
+        <v>XkMKJCvJKBk</v>
       </c>
       <c r="AI56" t="str">
-        <v>Captivating Nature Birds in 4K Ultra HD - A Visual Symphony of Wildlife Beauty</v>
+        <v>The History and Evolution of Citrus (Documentary)</v>
       </c>
       <c r="AJ56" t="str">
         <v>4K</v>
@@ -10525,7 +10525,7 @@
         <v>gbif | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM56" t="str">
-        <v>2026-08-01T15:19:32.777Z</v>
+        <v>2026-08-01T16:57:48.696Z</v>
       </c>
       <c r="AN56">
         <v>0.94</v>
@@ -10573,16 +10573,16 @@
         <v>2961</v>
       </c>
       <c r="BC56">
-        <v>2700</v>
+        <v>1239</v>
       </c>
       <c r="BD56">
-        <v>1779</v>
+        <v>929</v>
       </c>
       <c r="BE56" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF56" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>http://creativecommons.org/publicdomain/zero/1.0/deed.en</v>
       </c>
       <c r="BG56" t="str">
         <v>rights-free</v>
@@ -10680,22 +10680,22 @@
         <v/>
       </c>
       <c r="AD57" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/0/04/Favourite_flowers_of_garden_and_greenhouse_%2810593957506%29.jpg</v>
+        <v>https://upload.wikimedia.org/wikipedia/commons/e/e6/Amaranthus_tricolor_in_a_flower_bed_near_Notre-Dame_cathedral_in_Paris3.jpg</v>
       </c>
       <c r="AE57" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:Amaranthus_tricolor_by_Kakizaki_Hakyo_(Hakodate_City_Museum).jpg</v>
+        <v>https://commons.wikimedia.org/wiki/File:Amaranthus_tricolor_in_a_flower_bed_near_Notre-Dame_cathedral_in_Paris3.jpg</v>
       </c>
       <c r="AF57" t="str">
         <v>Public Domain</v>
       </c>
       <c r="AG57" t="str">
-        <v>https://www.youtube.com/watch?v=5Vu2bLQ5Gzs</v>
+        <v>https://www.youtube.com/watch?v=J62fxXP99yk</v>
       </c>
       <c r="AH57" t="str">
-        <v>5Vu2bLQ5Gzs</v>
+        <v>J62fxXP99yk</v>
       </c>
       <c r="AI57" t="str">
-        <v>3+ Hours of 4K Nature Adventures in Central America | FULL DOCUMENTARY | UHD | @UltimateNatureDocs</v>
+        <v>Amaranthus Tricolor Plant | Edible Amaranth | Nature Melody</v>
       </c>
       <c r="AJ57" t="str">
         <v>4K</v>
@@ -10707,7 +10707,7 @@
         <v>gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM57" t="str">
-        <v>2026-08-01T15:19:34.939Z</v>
+        <v>2026-08-01T16:57:54.020Z</v>
       </c>
       <c r="AN57">
         <v>0.99</v>
@@ -10755,13 +10755,13 @@
         <v/>
       </c>
       <c r="BC57">
-        <v>3643</v>
+        <v>2112</v>
       </c>
       <c r="BD57">
-        <v>2601</v>
+        <v>2816</v>
       </c>
       <c r="BE57" t="str">
-        <v>HD</v>
+        <v>Full HD</v>
       </c>
       <c r="BF57" t="str">
         <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
@@ -10862,22 +10862,22 @@
         <v/>
       </c>
       <c r="AD58" t="str">
-        <v>https://upload.wikimedia.org/wikipedia/commons/c/cb/Flore_des_serres_v15_141a.jpg</v>
+        <v>https://inaturalist-open-data.s3.amazonaws.com/photos/599773348/original.jpg</v>
       </c>
       <c r="AE58" t="str">
-        <v>https://commons.wikimedia.org/wiki/File:The_American_Flora._Vol._3,_1855_-_pl._01_Chrysanthemum_indicum_(10172162765).jpg</v>
+        <v>https://www.inaturalist.org/photos/599773348</v>
       </c>
       <c r="AF58" t="str">
-        <v>Public Domain</v>
+        <v>CC0</v>
       </c>
       <c r="AG58" t="str">
-        <v>https://www.youtube.com/watch?v=1DenEHzSU0c</v>
+        <v>https://www.youtube.com/watch?v=Kc_bKEuXYdw</v>
       </c>
       <c r="AH58" t="str">
-        <v>1DenEHzSU0c</v>
+        <v>Kc_bKEuXYdw</v>
       </c>
       <c r="AI58" t="str">
-        <v>Wildlife Wonders You’ve Never Seen Before | 4K Nature Documentary</v>
+        <v>Colorful Chrysanthemums Bloom with Birdsong | Nature Relaxation Flower Video #Chrysanthemum #Flowers</v>
       </c>
       <c r="AJ58" t="str">
         <v>4K</v>
@@ -10889,7 +10889,7 @@
         <v>gbif | wikipedia-en | wikipedia-vi | wikimedia | youtube | inaturalist</v>
       </c>
       <c r="AM58" t="str">
-        <v>2026-08-01T15:19:37.576Z</v>
+        <v>2026-08-01T16:57:59.023Z</v>
       </c>
       <c r="AN58">
         <v>0.97</v>
@@ -10937,16 +10937,16 @@
         <v/>
       </c>
       <c r="BC58">
-        <v>3264</v>
+        <v>2048</v>
       </c>
       <c r="BD58">
-        <v>2448</v>
+        <v>1536</v>
       </c>
       <c r="BE58" t="str">
         <v>Full HD</v>
       </c>
       <c r="BF58" t="str">
-        <v>https://creativecommons.org/publicdomain/mark/1.0/</v>
+        <v>https://creativecommons.org/publicdomain/zero/1.0/</v>
       </c>
       <c r="BG58" t="str">
         <v>rights-free</v>

</xml_diff>